<commit_message>
fixed bug in the exel handler where the fields where wrong
</commit_message>
<xml_diff>
--- a/data/excel/roundtrip_test.xlsx
+++ b/data/excel/roundtrip_test.xlsx
@@ -415,16 +415,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Roundtrip Test Chart</t>
         </is>
@@ -524,37 +536,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>frame</t>
+          <t>Property</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>polygon</t>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>line_color</t>
+          <t>frame</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>#FF0000</t>
+          <t>polygon</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>fill_color</t>
+          <t>line_color</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -566,80 +578,92 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fill</t>
-        </is>
-      </c>
-      <c r="B4" t="b">
-        <v>1</v>
+          <t>fill_color</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>#FF0000</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>alpha</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0.4</v>
+          <t>fill</t>
+        </is>
+      </c>
+      <c r="B5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ring_count</t>
+          <t>alpha</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>frame_width</t>
+          <t>ring_count</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>grid_width</t>
+          <t>frame_width</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>label_distance</t>
+          <t>grid_width</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>scale_label_offset</t>
+          <t>label_distance</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.03</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>scale_label_offset</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>grid_alpha</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B12" t="n">
         <v>0.3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Feature: editor now can load exel files and save the star charts
</commit_message>
<xml_diff>
--- a/data/excel/roundtrip_test.xlsx
+++ b/data/excel/roundtrip_test.xlsx
@@ -453,13 +453,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>label / meta</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -476,52 +476,99 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Angriff</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>80</v>
-      </c>
-      <c r="C2" t="n">
-        <v>60</v>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>#007ACC</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>#007ACC</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Verteidigung</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>90</v>
-      </c>
-      <c r="C3" t="n">
-        <v>75</v>
+          <t>marker</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tempo</t>
+          <t>line_width</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>70</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>85</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Angriff</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>80</v>
+      </c>
+      <c r="C5" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Verteidigung</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>90</v>
+      </c>
+      <c r="C6" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>70</v>
+      </c>
+      <c r="C7" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Ausdauer</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B8" t="n">
         <v>85</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C8" t="n">
         <v>70</v>
       </c>
     </row>
@@ -536,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -667,6 +714,16 @@
         <v>0.3</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>dpi</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>300</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>